<commit_message>
Update import template, change display text
</commit_message>
<xml_diff>
--- a/public/Ananbay_template.xlsx
+++ b/public/Ananbay_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28730"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\VSCode\TebGroup\teb-express-tunghoang\public\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\VSCode\TebGroup\aTung-tebexpress-cus\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39247435-F6B7-44F9-91D4-1FC35F3080D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{877A5DAD-B87D-4855-921A-95FA359540C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -149,22 +149,22 @@
     <t>Mã nhãn Tiktok</t>
   </si>
   <si>
-    <t>Express</t>
-  </si>
-  <si>
     <t>321075232</t>
   </si>
   <si>
     <t>321186905</t>
   </si>
   <si>
-    <t>https://seller-us.tiktok.com/wsos_v2/oec_fulfillment_doc_tts/object/wsos67e648f023c08b2b?expire=1743231678&amp;skipCookie=true&amp;timeStamp=1743145278&amp;sign=ec6024dfc8a63c6ee6d987234503f0f730fe44c15cc06b2757363a40d2a2c9b4</t>
-  </si>
-  <si>
     <t>Ship By Tiktok</t>
   </si>
   <si>
     <t>Hàng TradeMark</t>
+  </si>
+  <si>
+    <t>Standard</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/uc?export=download&amp;id=1gTk2GJUmt2k9FGdCRib01Qw9oOTSc0QU</t>
   </si>
 </sst>
 </file>
@@ -647,7 +647,7 @@
         <v>14</v>
       </c>
       <c r="P1" s="9" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="Q1" s="1" t="s">
         <v>15</v>
@@ -689,7 +689,7 @@
         <v>23</v>
       </c>
       <c r="I2" s="11" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="J2" s="7" t="s">
         <v>24</v>
@@ -707,7 +707,7 @@
         <v>3</v>
       </c>
       <c r="O2" s="7" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="P2" s="13" t="s">
         <v>26</v>
@@ -732,7 +732,7 @@
       <c r="G3" s="6"/>
       <c r="H3" s="3"/>
       <c r="I3" s="11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J3" s="7" t="s">
         <v>24</v>
@@ -750,11 +750,11 @@
         <v>3</v>
       </c>
       <c r="O3" s="7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="P3" s="13"/>
       <c r="R3" s="14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="S3" s="13" t="s">
         <v>26</v>
@@ -3383,7 +3383,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O519:O1048576" xr:uid="{10C1B1BA-30A4-43AA-B6F4-A5F0B0F55982}">
       <formula1>"Express, Tiktok"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S5:S6 S8:S1048576 S2:S3" xr:uid="{F8BCA374-D361-4313-9C59-CF82877BB18A}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S8:S1048576 S2:S6" xr:uid="{F8BCA374-D361-4313-9C59-CF82877BB18A}">
       <formula1>", YES, NO"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q5:Q1048576 Q2:Q3 P2:P520" xr:uid="{16DEDA22-1651-49B2-AAF1-65C50FFEDD2D}">
@@ -3392,13 +3392,10 @@
     <dataValidation type="custom" showInputMessage="1" showErrorMessage="1" sqref="R5:R526 R2:R3" xr:uid="{AB023EC7-7443-46B0-A956-FA2A83A11DFD}">
       <formula1>IF($O2="Tiktok", R2&lt;&gt;"", TRUE)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O2:O518" xr:uid="{8664190F-EA7C-4D2F-AC04-A222D6E43D96}">
-      <formula1>"Express, Ship By Tiktok"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O2:O518" xr:uid="{D4F5877A-3FE9-4602-ABFD-C44BAAB259EC}">
+      <formula1>"Standard, Express, Ship By Tiktok, Super Express"</formula1>
     </dataValidation>
   </dataValidations>
-  <hyperlinks>
-    <hyperlink ref="R3" r:id="rId1" xr:uid="{1BA6FB39-2A12-4199-9359-4A92E9981534}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>

</xml_diff>